<commit_message>
Fix UI buttons, session logout loop, add PDF invoice export without signatures, and sync Haj Salah invoice
</commit_message>
<xml_diff>
--- a/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
+++ b/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -734,126 +734,149 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>فاتورة 27 / 10</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>7326</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>ترابيع سيلفيا منها 28 صندوق</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>الاجمالي</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="9">
-        <f>SUM(C5:C8)</f>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="9">
+        <f>SUM(C5:C9)</f>
         <v/>
       </c>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>بيان الدفعة الواصلة</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>المبلغ (ج.م)</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>طريقة الدفع</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>واصل منه</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>نقداً</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>واصل منه</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>نقداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>واصل منه</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C14" s="6" t="n">
         <v>132500</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>نقداً</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>إجمالي الواصل منه</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="9">
-        <f>SUM(C12:C13)</f>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="9">
+        <f>SUM(C13:C14)</f>
         <v/>
       </c>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>المتبقي (الصافي المطلوب)</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="13">
-        <f>C9-C14</f>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="13">
+        <f>C10-C15</f>
         <v/>
       </c>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix auth (add missing login/logout functions to app.js), correct invoice 27/10 calculation: 28 boxes x 220 tiles = 6160 tiles, 1108.80 m2, total 205,128 EGP
</commit_message>
<xml_diff>
--- a/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
+++ b/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -232,6 +232,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -598,7 +599,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -743,7 +744,7 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>7326</v>
+        <v>205128</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -752,7 +753,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ترابيع سيلفيا منها 28 صندوق</t>
+          <t>ترابيع سيلفيا 28 صندوق × 220 تربيعة</t>
         </is>
       </c>
     </row>
@@ -762,7 +763,7 @@
           <t>الاجمالي</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
+      <c r="B10" s="23" t="n"/>
       <c r="C10" s="9">
         <f>SUM(C5:C9)</f>
         <v/>
@@ -849,7 +850,7 @@
           <t>إجمالي الواصل منه</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
+      <c r="B15" s="23" t="n"/>
       <c r="C15" s="9">
         <f>SUM(C13:C14)</f>
         <v/>
@@ -863,7 +864,7 @@
           <t>المتبقي (الصافي المطلوب)</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n"/>
+      <c r="B17" s="23" t="n"/>
       <c r="C17" s="13">
         <f>C10-C15</f>
         <v/>
@@ -873,10 +874,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -889,7 +890,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1017,7 +1018,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Update master ledger and Invoice 90 to match user reference photos exactly (327,393.43 EGP & 988,075.29 EGP remaining)
</commit_message>
<xml_diff>
--- a/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
+++ b/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="كشف الحساب المطور 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="كشف الحساب" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,12 +29,7 @@
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Cairo"/>
-      <color rgb="0064748B"/>
-      <sz val="11"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
@@ -44,20 +39,20 @@
     </font>
     <font>
       <name val="Cairo"/>
-      <b val="1"/>
+      <color rgb="000F172A"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="13"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00B91C1C"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -75,20 +70,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE7F3"/>
-        <bgColor rgb="00FCE7F3"/>
+        <fgColor rgb="00FEF08A"/>
+        <bgColor rgb="00FEF08A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="0015803D"/>
+        <bgColor rgb="0015803D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF08A"/>
-        <bgColor rgb="00FEF08A"/>
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,43 +113,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,340 +512,352 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>كشف حساب وسجل حركات: الحاج صلاح (النسخة المطورة 2026)</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>شركة ومصانع خالي أحمد جلال للرخام والجرانيت - إدارة الحسابات العامة</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
           <t>م</t>
         </is>
       </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>بيان الفاتورة</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>المبلغ (ج.م)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ملاحظات وتفاصيل التوريد</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 11 / 10</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>122828</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>11/10/2026</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>طاولة صني 3 سم (744.41 م٢) 137</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>بيان الفاتورة</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+          <t>فاتورة 23 / 9 (2)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>122755</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>23/9/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>طاولة صني 3 سم (743.90 م٢) 138</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 23 / 9 (1)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>121755</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>23/9/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>طاولة صني 3 سم (737.90 م٢) 133</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 3 / 10</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>125242</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>3/10/2026</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>طاولة سيلفيا 3 سم (659.17 م٢) 141</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 27 / 10 (1)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>205128</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>صندوق ترابيع سيلفيا = 6,160 تربيعة (1,108.80 م٢) 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 26 / 10 (1)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>122985.05</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>طاولة صني 3 سم (745.36 م٢) 132</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 26 / 10 (2)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>122488.81</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>طاولة صني 3 سم (742.36 م٢) 132</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>فاتورة 27 / 10 (2)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>327393.43</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>جرانيت (رويال 470 + جندولة 480 + نيوحلايب 355) + 3 شرائح رويال فري + سيلفيا 3 سم (40 طاولة @ 190)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="6" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>إجمالي المسحوبات (الفواتير)</t>
+        </is>
+      </c>
+      <c r="C11" s="8">
+        <f>SUM(C3:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>بيان الدفعة الواصلة</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>المبلغ (ج.م)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ملاحظات وتفاصيل التوريد</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>طريقة الدفع</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 11 / 10</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>122828</v>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>11/10/2026</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>137 قطعة (744.41 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>واصل منه</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>نقداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 23 / 9 (2)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>122755</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>23/9/2026</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>138 قطعة (743.90 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 23 / 9 (1)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>121755</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>23/9/2026</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>133 قطعة (737.90 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 3 / 10</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>125242</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>3/10/2026</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>141 قطعة (659.17 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 27 / 10</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>205128</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>6,160 قطعة (1,108.80 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 26 / 10 (1)</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>122985.05</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>132 قطعة (745.36 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>فاتورة 26 / 10 (2)</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>122488.81</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>132 قطعة (742.36 م٢)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>إجمالي المسحوبات (الفواتير)</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="9">
-        <f>SUM(C5:C11)</f>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>واصل منه</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>132500</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>نقداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="6" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>إجمالي الواصل منه (السدادات)</t>
+        </is>
+      </c>
+      <c r="C16" s="8">
+        <f>SUM(C14:C15)</f>
         <v/>
       </c>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>م</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>بيان الدفعة الواصلة</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>المبلغ (ج.م)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>طريقة الدفع</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>واصل منه</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>نقداً</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>واصل منه</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>132500</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>نقداً</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>إجمالي الواصل منه (السدادات)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="11">
-        <f>SUM(C15:C16)</f>
+      <c r="D16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>المتبقي (الصافي المطلوب)</t>
+        </is>
+      </c>
+      <c r="C18" s="12">
+        <f>C11-C16</f>
         <v/>
       </c>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>المتبقي (الصافي المطلوب)</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="13">
-        <f>C12-C17</f>
-        <v/>
-      </c>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A19:B19"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Haj Salah invoices 26-10 (1) and (2) with verified net dimensions and recalculate total ledger to 967,404.75 EGP
</commit_message>
<xml_diff>
--- a/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
+++ b/bundled_files/الحاج صلاح/حساب الحاج صلاح - النسخة المطورة 2026.xlsx
@@ -52,7 +52,7 @@
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00B91C1C"/>
-      <sz val="13"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="6">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>122985.05</v>
+        <v>112662.81</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>طاولة صني 3 سم (745.36 م٢) 132</t>
+          <t>طاولة صني 3 سم (682.81 م٢) 132</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>122488.81</v>
+        <v>112140.51</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>طاولة صني 3 سم (742.36 م٢) 132</t>
+          <t>طاولة صني 3 سم (679.64 م٢) 132</t>
         </is>
       </c>
     </row>

</xml_diff>